<commit_message>
update district heating bugs
fix bugs on spine importer, still bug in the python data prep
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/methanol/Model_Data_Base_methanol.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/methanol/Model_Data_Base_methanol.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\methanol\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\methanol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976B75BF-2265-4260-B68E-9D163759AD3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4C17597-52A4-42D8-B775-A7FB5182AF94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="126">
   <si>
     <t>Unit</t>
   </si>
@@ -352,21 +352,9 @@
     <t>initial_units_on</t>
   </si>
   <si>
-    <t>heat_low</t>
-  </si>
-  <si>
-    <t>heat_high</t>
-  </si>
-  <si>
-    <t>heat_split</t>
-  </si>
-  <si>
     <t>Auxilliary</t>
   </si>
   <si>
-    <t>internal_heat</t>
-  </si>
-  <si>
     <t>Input3</t>
   </si>
   <si>
@@ -458,6 +446,12 @@
   </si>
   <si>
     <t>pl_wind_offshore_PPA</t>
+  </si>
+  <si>
+    <t>heat</t>
+  </si>
+  <si>
+    <t>excess_heat</t>
   </si>
 </sst>
 </file>
@@ -1287,8 +1281,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}" name="Table1" displayName="Table1" ref="A1:R12" totalsRowShown="0">
-  <autoFilter ref="A1:R12" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}" name="Table1" displayName="Table1" ref="A1:R11" totalsRowShown="0">
+  <autoFilter ref="A1:R11" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
   <tableColumns count="18">
     <tableColumn id="1" xr3:uid="{C73E51D0-1842-42F3-9C00-F0DBD2E661BE}" name="Unit"/>
     <tableColumn id="40" xr3:uid="{C2CFC5A4-5329-4F74-926A-18CEB18C062C}" name="Object_type"/>
@@ -1314,8 +1308,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}" name="Table5" displayName="Table5" ref="A1:Q12" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21" totalsRowBorderDxfId="20">
-  <autoFilter ref="A1:Q12" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}" name="Table5" displayName="Table5" ref="A1:Q11" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21" totalsRowBorderDxfId="20">
+  <autoFilter ref="A1:Q11" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{2BE3E317-773B-4E82-9035-69A43C6CB21B}" name="Unit" dataDxfId="19"/>
     <tableColumn id="2" xr3:uid="{22613EE0-390D-4B04-9A9B-6D5554D1C8ED}" name="Object_type" dataDxfId="18"/>
@@ -1704,15 +1698,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576C757C-091A-46DF-949E-B17661031FDE}">
-  <dimension ref="A1:R12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="18" width="10.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="18" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1720,7 +1714,7 @@
         <v>43</v>
       </c>
       <c r="C1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
@@ -1729,16 +1723,16 @@
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="H1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="I1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="J1" t="s">
         <v>64</v>
@@ -1768,7 +1762,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -1776,38 +1770,38 @@
         <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B3" t="s">
         <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
         <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>89</v>
       </c>
@@ -1829,7 +1823,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1842,7 +1836,7 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>84</v>
       </c>
@@ -1859,7 +1853,7 @@
         <v>20.192799999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>83</v>
       </c>
@@ -1896,7 +1890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -1912,12 +1906,12 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C10" t="s">
         <v>75</v>
@@ -1925,36 +1919,23 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C11" t="s">
         <v>86</v>
       </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C12" t="s">
-        <v>93</v>
-      </c>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P12" xr:uid="{D92CB468-B7A9-4082-9B81-D3B4634F286E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P2:P11" xr:uid="{D92CB468-B7A9-4082-9B81-D3B4634F286E}">
       <formula1>"h, D, W, M, Q, Y"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1980,16 +1961,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CABA7C5-6230-4207-9D35-0A95D86E66AC}">
-  <dimension ref="A1:Q12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Q11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2003,10 +1984,10 @@
         <v>2</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>3</v>
@@ -2015,34 +1996,34 @@
         <v>4</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>69</v>
       </c>
@@ -2054,7 +2035,7 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="7"/>
@@ -2067,9 +2048,9 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>62</v>
@@ -2079,7 +2060,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -2092,9 +2073,9 @@
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
         <v>63</v>
@@ -2104,7 +2085,7 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -2117,7 +2098,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>89</v>
       </c>
@@ -2136,7 +2117,7 @@
         <v>78</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -2152,7 +2133,7 @@
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>85</v>
       </c>
@@ -2185,7 +2166,7 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>84</v>
       </c>
@@ -2219,7 +2200,7 @@
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>83</v>
       </c>
@@ -2237,8 +2218,8 @@
       <c r="G8" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>93</v>
+      <c r="H8" s="4" t="s">
+        <v>125</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
@@ -2257,7 +2238,7 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>77</v>
       </c>
@@ -2290,94 +2271,63 @@
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="H10" s="6" t="s">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6">
+      <c r="C10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4">
         <v>1</v>
       </c>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4">
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+      <c r="Q10" s="4"/>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6">
         <v>1</v>
       </c>
-      <c r="O11" s="4"/>
-      <c r="P11" s="4"/>
-      <c r="Q11" s="4"/>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6">
-        <v>1</v>
-      </c>
-      <c r="O12" s="6"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
+      <c r="Q11" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -2392,7 +2342,7 @@
           <x14:formula1>
             <xm:f>Drop_Down!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>B1:B12</xm:sqref>
+          <xm:sqref>B1:B11</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2403,34 +2353,34 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C870BDA0-9E4C-481D-87BE-9D47789809C8}">
   <dimension ref="A1:AA11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" customWidth="1"/>
-    <col min="9" max="9" width="17.42578125" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" customWidth="1"/>
-    <col min="11" max="11" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" customWidth="1"/>
+    <col min="7" max="7" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.33203125" customWidth="1"/>
+    <col min="9" max="9" width="17.44140625" customWidth="1"/>
+    <col min="10" max="10" width="15.44140625" customWidth="1"/>
+    <col min="11" max="11" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" customWidth="1"/>
     <col min="13" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" customWidth="1"/>
+    <col min="14" max="14" width="15.44140625" customWidth="1"/>
     <col min="15" max="15" width="19" customWidth="1"/>
-    <col min="16" max="16" width="10.5703125" customWidth="1"/>
-    <col min="17" max="17" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.7109375" customWidth="1"/>
-    <col min="21" max="21" width="12.7109375" customWidth="1"/>
-    <col min="22" max="23" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.5546875" customWidth="1"/>
+    <col min="17" max="17" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.6640625" customWidth="1"/>
+    <col min="21" max="21" width="12.6640625" customWidth="1"/>
+    <col min="22" max="23" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -2513,7 +2463,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>71</v>
       </c>
@@ -2572,7 +2522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>88</v>
       </c>
@@ -2628,7 +2578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>90</v>
       </c>
@@ -2684,7 +2634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -2692,7 +2642,7 @@
         <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>124</v>
       </c>
       <c r="E5" t="s">
         <v>74</v>
@@ -2722,9 +2672,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B6" t="s">
         <v>53</v>
@@ -2733,10 +2683,10 @@
         <v>72</v>
       </c>
       <c r="D6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F6" t="s">
         <v>72</v>
@@ -2781,15 +2731,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B7" t="s">
         <v>53</v>
       </c>
       <c r="C7" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E7" t="s">
         <v>70</v>
@@ -2819,9 +2769,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B8" t="s">
         <v>53</v>
@@ -2830,10 +2780,10 @@
         <v>72</v>
       </c>
       <c r="D8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F8" t="s">
         <v>72</v>
@@ -2878,15 +2828,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B9" t="s">
         <v>53</v>
       </c>
       <c r="C9" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E9" t="s">
         <v>70</v>
@@ -2916,9 +2866,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B10" t="s">
         <v>53</v>
@@ -2927,10 +2877,10 @@
         <v>72</v>
       </c>
       <c r="D10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F10" t="s">
         <v>72</v>
@@ -2975,15 +2925,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B11" t="s">
         <v>53</v>
       </c>
       <c r="C11" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E11" t="s">
         <v>70</v>
@@ -3038,22 +2988,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{981CFA5E-60F3-446F-A856-2FA65B76879A}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.28515625" customWidth="1"/>
+    <col min="10" max="10" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -3088,7 +3038,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -3114,7 +3064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -3169,104 +3119,104 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DC79B9-9C58-497E-9FD8-D3F2239E9BDC}">
   <dimension ref="A1:A19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>